<commit_message>
Adiciona 28 produtos manuais (SUVINIL, BLASCOR, CORAL, COLORGIN etc.) na lista RT oficial
</commit_message>
<xml_diff>
--- a/data/lista_produtos_RToficial.xlsx
+++ b/data/lista_produtos_RToficial.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\souza\Documents\produtos omie 21092026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AC68746-403F-4864-A7CE-A9F7F521C76A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8F0A76B-75E1-45DB-8EA0-05F3200F1CFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20683" uniqueCount="3756">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20851" uniqueCount="3783">
   <si>
     <t>codigo</t>
   </si>
@@ -11297,6 +11297,87 @@
   </si>
   <si>
     <t>7730149548455</t>
+  </si>
+  <si>
+    <t>CORAL ADESIVO SELANTE PU 40 CINZA - ELASTIQUE 400G - MACTRA</t>
+  </si>
+  <si>
+    <t>manual</t>
+  </si>
+  <si>
+    <t>BLASCOR FUNDO PREPARADOR 3,6L</t>
+  </si>
+  <si>
+    <t>BLASCOR MASSA ACRÍLICA 3,6L</t>
+  </si>
+  <si>
+    <t>BLASCOR SELADOR ACRÍLICO 3,6 L</t>
+  </si>
+  <si>
+    <t>BRASILUX BASE EFEITO MARMORE GALAO 4 KG</t>
+  </si>
+  <si>
+    <t>BRAZILIAN MASSA ACRILICA 1/4</t>
+  </si>
+  <si>
+    <t>COLORGIN ALTA TEMP PRETO 350ML</t>
+  </si>
+  <si>
+    <t>COLORGIN DECOR SPRAY MULTIUSO 300ML CINZA</t>
+  </si>
+  <si>
+    <t>COLORGIN DECOR SPRAY MULTIUSO 300ML LARANJA</t>
+  </si>
+  <si>
+    <t>COLORGIN DECOR SPRAY MULTIUSO 300ML VERDE FOLHA</t>
+  </si>
+  <si>
+    <t>COLORGIN VERNIZ PLASTIC SPRAY  BRILHANTE 300ML</t>
+  </si>
+  <si>
+    <t>CORAL DECORA MATTE EXTRA FOSCO BASE MF 3,2L</t>
+  </si>
+  <si>
+    <t>CORAL SEDA ACET BASE MF 3,2L</t>
+  </si>
+  <si>
+    <t>AEROFLEX DESINGRIPANTE LUBRIFICANTE AEROSOL 300ML LUB FAST</t>
+  </si>
+  <si>
+    <t>BRAZILIAN EPÓXI CINZA M N3,5 COLORSTEEL 2,7 L</t>
+  </si>
+  <si>
+    <t>BRAZILIAN EPÓXI VERMELHO SEGURANÇA 5R 4/14</t>
+  </si>
+  <si>
+    <t>EUROCEL FITA ADESIVA PARA DEMARCAÇÃO DE SOLO 50MM X 15M</t>
+  </si>
+  <si>
+    <t>BLASCOR MASSA ACRILICA 1,45 KG</t>
+  </si>
+  <si>
+    <t>SIKA SELANTE ACR P/FENDA TRINCA CARTUCHO 280ML 430G SIKAKRYL 203 6610</t>
+  </si>
+  <si>
+    <t>UNIPEGA SELANTE PU FLEX  UNIPEGA BRANCO 280ML</t>
+  </si>
+  <si>
+    <t>MUNDIAL PRIME SELANTE PU40 PRETO 400G MUNDIAL PRIME</t>
+  </si>
+  <si>
+    <t>QUIMATIC TAPMATIC SPRAY GALVAMULE FUNDO GAVANIZAÇÃO 300ML</t>
+  </si>
+  <si>
+    <t>SUVINIL EPOXI MULTISUPERFÍCIES BASE A 800ML ACETINADO</t>
+  </si>
+  <si>
+    <t>SUVINIL EPOXI MULTISUPERFÍCIES BASE B 800ML ACETINADO</t>
+  </si>
+  <si>
+    <t>SUVINIL EPOXI MULTISUPERFÍCIES BASE C 800ML ACETINADO</t>
+  </si>
+  <si>
+    <t>SUVINIL TOQUE COMPLETO FOSCO BRANCO NEVE 900ML</t>
   </si>
 </sst>
 </file>
@@ -11636,7 +11717,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K968"/>
+  <dimension ref="A1:K996"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
@@ -40034,6 +40115,818 @@
       </c>
       <c r="K968" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="969" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A969">
+        <v>7897866466063</v>
+      </c>
+      <c r="B969" t="s">
+        <v>3756</v>
+      </c>
+      <c r="C969">
+        <v>7897866466063</v>
+      </c>
+      <c r="D969">
+        <v>7897866466063</v>
+      </c>
+      <c r="E969" t="s">
+        <v>18</v>
+      </c>
+      <c r="F969" t="s">
+        <v>5</v>
+      </c>
+      <c r="G969" t="s">
+        <v>18</v>
+      </c>
+      <c r="H969" t="s">
+        <v>0</v>
+      </c>
+      <c r="K969" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="970" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A970">
+        <v>7898514580797</v>
+      </c>
+      <c r="B970" t="s">
+        <v>3758</v>
+      </c>
+      <c r="C970">
+        <v>7898514580797</v>
+      </c>
+      <c r="D970">
+        <v>7898514580797</v>
+      </c>
+      <c r="E970" t="s">
+        <v>18</v>
+      </c>
+      <c r="F970" t="s">
+        <v>5</v>
+      </c>
+      <c r="G970" t="s">
+        <v>18</v>
+      </c>
+      <c r="H970" t="s">
+        <v>0</v>
+      </c>
+      <c r="K970" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="971" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A971">
+        <v>7898514580056</v>
+      </c>
+      <c r="B971" t="s">
+        <v>3759</v>
+      </c>
+      <c r="C971">
+        <v>7898514580056</v>
+      </c>
+      <c r="D971">
+        <v>7898514580056</v>
+      </c>
+      <c r="E971" t="s">
+        <v>18</v>
+      </c>
+      <c r="F971" t="s">
+        <v>5</v>
+      </c>
+      <c r="G971" t="s">
+        <v>18</v>
+      </c>
+      <c r="H971" t="s">
+        <v>0</v>
+      </c>
+      <c r="K971" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="972" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A972">
+        <v>4137074580315</v>
+      </c>
+      <c r="B972" t="s">
+        <v>3760</v>
+      </c>
+      <c r="C972">
+        <v>4137074580315</v>
+      </c>
+      <c r="D972">
+        <v>4137074580315</v>
+      </c>
+      <c r="E972" t="s">
+        <v>18</v>
+      </c>
+      <c r="F972" t="s">
+        <v>5</v>
+      </c>
+      <c r="G972" t="s">
+        <v>18</v>
+      </c>
+      <c r="H972" t="s">
+        <v>0</v>
+      </c>
+      <c r="K972" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="973" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A973">
+        <v>7893866083569</v>
+      </c>
+      <c r="B973" t="s">
+        <v>3761</v>
+      </c>
+      <c r="C973">
+        <v>7893866083569</v>
+      </c>
+      <c r="D973">
+        <v>7893866083569</v>
+      </c>
+      <c r="E973" t="s">
+        <v>18</v>
+      </c>
+      <c r="F973" t="s">
+        <v>5</v>
+      </c>
+      <c r="G973" t="s">
+        <v>18</v>
+      </c>
+      <c r="H973" t="s">
+        <v>0</v>
+      </c>
+      <c r="K973" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="974" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A974">
+        <v>7899044752258</v>
+      </c>
+      <c r="B974" t="s">
+        <v>3762</v>
+      </c>
+      <c r="C974">
+        <v>7899044752258</v>
+      </c>
+      <c r="D974">
+        <v>7899044752258</v>
+      </c>
+      <c r="E974" t="s">
+        <v>18</v>
+      </c>
+      <c r="F974" t="s">
+        <v>5</v>
+      </c>
+      <c r="G974" t="s">
+        <v>18</v>
+      </c>
+      <c r="H974" t="s">
+        <v>0</v>
+      </c>
+      <c r="K974" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="975" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A975">
+        <v>7891494057228</v>
+      </c>
+      <c r="B975" t="s">
+        <v>3763</v>
+      </c>
+      <c r="C975">
+        <v>7891494057228</v>
+      </c>
+      <c r="D975">
+        <v>7891494057228</v>
+      </c>
+      <c r="E975" t="s">
+        <v>18</v>
+      </c>
+      <c r="F975" t="s">
+        <v>5</v>
+      </c>
+      <c r="G975" t="s">
+        <v>18</v>
+      </c>
+      <c r="H975" t="s">
+        <v>0</v>
+      </c>
+      <c r="K975" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="976" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A976">
+        <v>7891494086518</v>
+      </c>
+      <c r="B976" t="s">
+        <v>3764</v>
+      </c>
+      <c r="C976">
+        <v>7891494086518</v>
+      </c>
+      <c r="D976">
+        <v>7891494086518</v>
+      </c>
+      <c r="E976" t="s">
+        <v>18</v>
+      </c>
+      <c r="F976" t="s">
+        <v>5</v>
+      </c>
+      <c r="G976" t="s">
+        <v>18</v>
+      </c>
+      <c r="H976" t="s">
+        <v>0</v>
+      </c>
+      <c r="K976" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="977" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A977">
+        <v>7891494088314</v>
+      </c>
+      <c r="B977" t="s">
+        <v>3765</v>
+      </c>
+      <c r="C977">
+        <v>7891494088314</v>
+      </c>
+      <c r="D977">
+        <v>7891494088314</v>
+      </c>
+      <c r="E977" t="s">
+        <v>18</v>
+      </c>
+      <c r="F977" t="s">
+        <v>5</v>
+      </c>
+      <c r="G977" t="s">
+        <v>18</v>
+      </c>
+      <c r="H977" t="s">
+        <v>0</v>
+      </c>
+      <c r="K977" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="978" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A978">
+        <v>7891494087515</v>
+      </c>
+      <c r="B978" t="s">
+        <v>3766</v>
+      </c>
+      <c r="C978">
+        <v>7891494087515</v>
+      </c>
+      <c r="D978">
+        <v>7891494087515</v>
+      </c>
+      <c r="E978" t="s">
+        <v>18</v>
+      </c>
+      <c r="F978" t="s">
+        <v>5</v>
+      </c>
+      <c r="G978" t="s">
+        <v>18</v>
+      </c>
+      <c r="H978" t="s">
+        <v>0</v>
+      </c>
+      <c r="K978" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="979" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A979">
+        <v>7891494007803</v>
+      </c>
+      <c r="B979" t="s">
+        <v>3767</v>
+      </c>
+      <c r="C979">
+        <v>7891494007803</v>
+      </c>
+      <c r="D979">
+        <v>7891494007803</v>
+      </c>
+      <c r="E979" t="s">
+        <v>18</v>
+      </c>
+      <c r="F979" t="s">
+        <v>5</v>
+      </c>
+      <c r="G979" t="s">
+        <v>18</v>
+      </c>
+      <c r="H979" t="s">
+        <v>0</v>
+      </c>
+      <c r="K979" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="980" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A980">
+        <v>7891019022137</v>
+      </c>
+      <c r="B980" t="s">
+        <v>3768</v>
+      </c>
+      <c r="C980">
+        <v>7891019022137</v>
+      </c>
+      <c r="D980">
+        <v>7891019022137</v>
+      </c>
+      <c r="E980" t="s">
+        <v>18</v>
+      </c>
+      <c r="F980" t="s">
+        <v>5</v>
+      </c>
+      <c r="G980" t="s">
+        <v>18</v>
+      </c>
+      <c r="H980" t="s">
+        <v>0</v>
+      </c>
+      <c r="K980" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="981" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A981">
+        <v>7891019022335</v>
+      </c>
+      <c r="B981" t="s">
+        <v>3769</v>
+      </c>
+      <c r="C981">
+        <v>7891019022335</v>
+      </c>
+      <c r="D981">
+        <v>7891019022335</v>
+      </c>
+      <c r="E981" t="s">
+        <v>18</v>
+      </c>
+      <c r="F981" t="s">
+        <v>5</v>
+      </c>
+      <c r="G981" t="s">
+        <v>18</v>
+      </c>
+      <c r="H981" t="s">
+        <v>0</v>
+      </c>
+      <c r="K981" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="982" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A982">
+        <v>7898567700944</v>
+      </c>
+      <c r="B982" t="s">
+        <v>3770</v>
+      </c>
+      <c r="C982">
+        <v>7898567700944</v>
+      </c>
+      <c r="D982">
+        <v>7898567700944</v>
+      </c>
+      <c r="E982" t="s">
+        <v>18</v>
+      </c>
+      <c r="F982" t="s">
+        <v>5</v>
+      </c>
+      <c r="G982" t="s">
+        <v>18</v>
+      </c>
+      <c r="H982" t="s">
+        <v>0</v>
+      </c>
+      <c r="K982" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="983" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A983">
+        <v>7899044758564</v>
+      </c>
+      <c r="B983" t="s">
+        <v>3771</v>
+      </c>
+      <c r="C983">
+        <v>7899044758564</v>
+      </c>
+      <c r="D983">
+        <v>7899044758564</v>
+      </c>
+      <c r="E983" t="s">
+        <v>18</v>
+      </c>
+      <c r="F983" t="s">
+        <v>5</v>
+      </c>
+      <c r="G983" t="s">
+        <v>18</v>
+      </c>
+      <c r="H983" t="s">
+        <v>0</v>
+      </c>
+      <c r="K983" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="984" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A984">
+        <v>7899044756034</v>
+      </c>
+      <c r="B984" t="s">
+        <v>3772</v>
+      </c>
+      <c r="C984">
+        <v>7899044756034</v>
+      </c>
+      <c r="D984">
+        <v>7899044756034</v>
+      </c>
+      <c r="E984" t="s">
+        <v>18</v>
+      </c>
+      <c r="F984" t="s">
+        <v>5</v>
+      </c>
+      <c r="G984" t="s">
+        <v>18</v>
+      </c>
+      <c r="H984" t="s">
+        <v>0</v>
+      </c>
+      <c r="K984" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="985" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A985">
+        <v>7899320356408</v>
+      </c>
+      <c r="B985" t="s">
+        <v>3773</v>
+      </c>
+      <c r="C985">
+        <v>7899320356408</v>
+      </c>
+      <c r="D985">
+        <v>7899320356408</v>
+      </c>
+      <c r="E985" t="s">
+        <v>18</v>
+      </c>
+      <c r="F985" t="s">
+        <v>5</v>
+      </c>
+      <c r="G985" t="s">
+        <v>18</v>
+      </c>
+      <c r="H985" t="s">
+        <v>0</v>
+      </c>
+      <c r="K985" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="986" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A986">
+        <v>7899763105342</v>
+      </c>
+      <c r="B986" t="s">
+        <v>3774</v>
+      </c>
+      <c r="C986">
+        <v>7899763105342</v>
+      </c>
+      <c r="D986">
+        <v>7899763105342</v>
+      </c>
+      <c r="E986" t="s">
+        <v>18</v>
+      </c>
+      <c r="F986" t="s">
+        <v>5</v>
+      </c>
+      <c r="G986" t="s">
+        <v>18</v>
+      </c>
+      <c r="H986" t="s">
+        <v>0</v>
+      </c>
+      <c r="K986" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="987" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A987">
+        <v>7896785315483</v>
+      </c>
+      <c r="B987" t="s">
+        <v>3775</v>
+      </c>
+      <c r="C987">
+        <v>7896785315483</v>
+      </c>
+      <c r="D987">
+        <v>7896785315483</v>
+      </c>
+      <c r="E987" t="s">
+        <v>18</v>
+      </c>
+      <c r="F987" t="s">
+        <v>5</v>
+      </c>
+      <c r="G987" t="s">
+        <v>18</v>
+      </c>
+      <c r="H987" t="s">
+        <v>0</v>
+      </c>
+      <c r="K987" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="988" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A988">
+        <v>7898652120428</v>
+      </c>
+      <c r="B988" t="s">
+        <v>3776</v>
+      </c>
+      <c r="C988">
+        <v>7898652120428</v>
+      </c>
+      <c r="D988">
+        <v>7898652120428</v>
+      </c>
+      <c r="E988" t="s">
+        <v>18</v>
+      </c>
+      <c r="F988" t="s">
+        <v>5</v>
+      </c>
+      <c r="G988" t="s">
+        <v>18</v>
+      </c>
+      <c r="H988" t="s">
+        <v>0</v>
+      </c>
+      <c r="K988" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="989" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A989">
+        <v>7898567703624</v>
+      </c>
+      <c r="B989" t="s">
+        <v>3777</v>
+      </c>
+      <c r="C989">
+        <v>7898567703624</v>
+      </c>
+      <c r="D989">
+        <v>7898567703624</v>
+      </c>
+      <c r="E989" t="s">
+        <v>18</v>
+      </c>
+      <c r="F989" t="s">
+        <v>5</v>
+      </c>
+      <c r="G989" t="s">
+        <v>18</v>
+      </c>
+      <c r="H989" t="s">
+        <v>0</v>
+      </c>
+      <c r="K989" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="990" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A990">
+        <v>7898001616367</v>
+      </c>
+      <c r="B990" t="s">
+        <v>3778</v>
+      </c>
+      <c r="C990">
+        <v>7898001616367</v>
+      </c>
+      <c r="D990">
+        <v>7898001616367</v>
+      </c>
+      <c r="E990" t="s">
+        <v>18</v>
+      </c>
+      <c r="F990" t="s">
+        <v>5</v>
+      </c>
+      <c r="G990" t="s">
+        <v>18</v>
+      </c>
+      <c r="H990" t="s">
+        <v>0</v>
+      </c>
+      <c r="K990" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="991" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A991">
+        <v>7891260394410</v>
+      </c>
+      <c r="B991" t="s">
+        <v>3779</v>
+      </c>
+      <c r="C991">
+        <v>7891260394410</v>
+      </c>
+      <c r="D991">
+        <v>7891260394410</v>
+      </c>
+      <c r="E991" t="s">
+        <v>18</v>
+      </c>
+      <c r="F991" t="s">
+        <v>5</v>
+      </c>
+      <c r="G991" t="s">
+        <v>18</v>
+      </c>
+      <c r="H991" t="s">
+        <v>0</v>
+      </c>
+      <c r="K991" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="992" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A992">
+        <v>7891260561782</v>
+      </c>
+      <c r="B992" t="s">
+        <v>3780</v>
+      </c>
+      <c r="C992">
+        <v>7891260561782</v>
+      </c>
+      <c r="D992">
+        <v>7891260561782</v>
+      </c>
+      <c r="E992" t="s">
+        <v>18</v>
+      </c>
+      <c r="F992" t="s">
+        <v>5</v>
+      </c>
+      <c r="G992" t="s">
+        <v>18</v>
+      </c>
+      <c r="H992" t="s">
+        <v>0</v>
+      </c>
+      <c r="K992" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="993" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A993">
+        <v>7891260399972</v>
+      </c>
+      <c r="B993" t="s">
+        <v>3781</v>
+      </c>
+      <c r="C993">
+        <v>7891260399972</v>
+      </c>
+      <c r="D993">
+        <v>7891260399972</v>
+      </c>
+      <c r="E993" t="s">
+        <v>18</v>
+      </c>
+      <c r="F993" t="s">
+        <v>5</v>
+      </c>
+      <c r="G993" t="s">
+        <v>18</v>
+      </c>
+      <c r="H993" t="s">
+        <v>0</v>
+      </c>
+      <c r="K993" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="994" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A994">
+        <v>7891260560983</v>
+      </c>
+      <c r="B994" t="s">
+        <v>3659</v>
+      </c>
+      <c r="C994">
+        <v>7891260560983</v>
+      </c>
+      <c r="D994">
+        <v>7891260560983</v>
+      </c>
+      <c r="E994" t="s">
+        <v>18</v>
+      </c>
+      <c r="F994" t="s">
+        <v>5</v>
+      </c>
+      <c r="G994" t="s">
+        <v>18</v>
+      </c>
+      <c r="H994" t="s">
+        <v>0</v>
+      </c>
+      <c r="K994" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="995" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A995">
+        <v>7891260560877</v>
+      </c>
+      <c r="B995" t="s">
+        <v>2669</v>
+      </c>
+      <c r="C995">
+        <v>7891260560877</v>
+      </c>
+      <c r="D995">
+        <v>7891260560877</v>
+      </c>
+      <c r="E995" t="s">
+        <v>18</v>
+      </c>
+      <c r="F995" t="s">
+        <v>5</v>
+      </c>
+      <c r="G995" t="s">
+        <v>18</v>
+      </c>
+      <c r="H995" t="s">
+        <v>0</v>
+      </c>
+      <c r="K995" t="s">
+        <v>3757</v>
+      </c>
+    </row>
+    <row r="996" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A996">
+        <v>7891260560860</v>
+      </c>
+      <c r="B996" t="s">
+        <v>3782</v>
+      </c>
+      <c r="C996">
+        <v>7891260560860</v>
+      </c>
+      <c r="D996">
+        <v>7891260560860</v>
+      </c>
+      <c r="E996" t="s">
+        <v>18</v>
+      </c>
+      <c r="F996" t="s">
+        <v>5</v>
+      </c>
+      <c r="G996" t="s">
+        <v>18</v>
+      </c>
+      <c r="H996" t="s">
+        <v>0</v>
+      </c>
+      <c r="K996" t="s">
+        <v>3757</v>
       </c>
     </row>
   </sheetData>

</xml_diff>